<commit_message>
Gameplay: tune patch placement hitboxes
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/game_balance_sheet.xlsx
+++ b/game_balance_sheet.xlsx
@@ -284,7 +284,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:F21"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -330,33 +330,35 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PumpkinPatch</t>
+          <t>AppleTree</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Patch</t>
+          <t>Tree</t>
         </is>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
-      <c r="D2">
-        <v>1</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="E2">
         <f>IF(B2="Patch",C2*60/D2,C2*Assumptions!$B$3*60)</f>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>starter patch</t>
+          <t>starter tree</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CabbagePatch</t>
+          <t>PumpkinPatch</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -375,31 +377,33 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>early patch</t>
+          <t>second progression patch</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AppleTree</t>
+          <t>CabbagePatch</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Tree</t>
+          <t>Patch</t>
         </is>
       </c>
       <c r="C4">
         <v>2</v>
       </c>
-      <c r="D4"/>
+      <c r="D4">
+        <v>1</v>
+      </c>
       <c r="E4">
         <f>IF(B4="Patch",C4*60/D4,C4*Assumptions!$B$3*60)</f>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>tree fruit XP</t>
+          <t>third progression patch</t>
         </is>
       </c>
     </row>
@@ -763,7 +767,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:J54"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -857,7 +861,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>PumpkinPatch</t>
+          <t>AppleTree</t>
         </is>
       </c>
       <c r="H2">
@@ -899,7 +903,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>PumpkinPatch</t>
+          <t>AppleTree</t>
         </is>
       </c>
       <c r="H3">
@@ -941,7 +945,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>PumpkinPatch</t>
+          <t>AppleTree</t>
         </is>
       </c>
       <c r="H4">
@@ -983,7 +987,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>CabbagePatch</t>
+          <t>PumpkinPatch</t>
         </is>
       </c>
       <c r="H5">
@@ -1025,7 +1029,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>CabbagePatch</t>
+          <t>PumpkinPatch</t>
         </is>
       </c>
       <c r="H6">
@@ -1067,7 +1071,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>CabbagePatch</t>
+          <t>PumpkinPatch</t>
         </is>
       </c>
       <c r="H7">
@@ -1109,7 +1113,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>AppleTree</t>
+          <t>CabbagePatch</t>
         </is>
       </c>
       <c r="H8">
@@ -1151,7 +1155,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>AppleTree</t>
+          <t>CabbagePatch</t>
         </is>
       </c>
       <c r="H9">
@@ -3052,7 +3056,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:M21"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -3140,17 +3144,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PumpkinSeed</t>
+          <t>AppleTreeSeed</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Pumpkin Seed</t>
+          <t>Apple Tree Seed</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PumpkinPatch</t>
+          <t>AppleTree</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -3191,17 +3195,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CabbageSeed</t>
+          <t>PumpkinSeed</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cabbage Seed</t>
+          <t>Pumpkin Seed</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CabbagePatch</t>
+          <t>PumpkinPatch</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -3242,17 +3246,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AppleTreeSeed</t>
+          <t>CabbageSeed</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Apple Tree Seed</t>
+          <t>Cabbage Seed</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AppleTree</t>
+          <t>CabbagePatch</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">

</xml_diff>